<commit_message>
fix: start with channel#0
Breaking change:

initial code considered (f_max - f_min) / spacing for channel count in design,
but used (f_max - f_min) / spacing - 1 channels, for propagation, starting the propagation
with f_min + spacing and stopping at f_max.

This change aligns both design and propagation:
Number of channels is now the same for design and propagation for a given SI,
and channel numbers starts at f_min (included) and stop at f_max (included)

Signed-off-by: EstherLerouzic <esther.lerouzic@orange.com>
Change-Id: I8a6192bc26df0acd814186165807bffca08210ea
</commit_message>
<xml_diff>
--- a/tests/data/parser/transmission/results_transmission_multiband_expected.xlsx
+++ b/tests/data/parser/transmission/results_transmission_multiband_expected.xlsx
@@ -413,11 +413,11 @@
 		o Att in: 0 dB
 	band 186.500-190.100 THz
 		o Type: std_medium_gain_L
-		o Effective_gain (before att_in and before output VOA): 22.427 dB
+		o Effective_gain (before att_in and before output VOA): 22.367 dB
 		o P in: -1.487 dBm
-		o P out: 20.946 dBm
-		o P out/ch: -0.57 dBm
-		o NF: 6.17 dB
+		o P out: 20.887 dBm
+		o P out/ch: -0.63 dBm
+		o NF: 6.18 dB
 		o Out VOA: 3.0 dB
 		o In VOA: 0 dB
 		o Att in: 0 dB
@@ -454,9 +454,9 @@
 	band 186.500-190.100 THz
 		o Type: std_medium_gain_L
 		o Effective_gain (before att_in and before output VOA): 18.0 dB
-		o P in: 2.946 dBm
-		o P out: 20.95 dBm
-		o P out/ch: -0.56 dBm
+		o P in: 2.887 dBm
+		o P out: 20.89 dBm
+		o P out/ch: -0.62 dBm
 		o NF: 7.38 dB
 		o Out VOA: 3.0 dB
 		o In VOA: 0 dB
@@ -494,9 +494,9 @@
 	band 186.500-190.100 THz
 		o Type: std_medium_gain_L
 		o Effective_gain (before att_in and before output VOA): 19.8 dB
-		o P in: 1.15 dBm
-		o P out: 20.954 dBm
-		o P out/ch: -0.56 dBm
+		o P in: 1.09 dBm
+		o P out: 20.894 dBm
+		o P out/ch: -0.62 dBm
 		o NF: 6.63 dB
 		o Out VOA: 3.0 dB
 		o In VOA: 0 dB
@@ -534,9 +534,9 @@
 	band 186.500-190.100 THz
 		o Type: std_medium_gain_L
 		o Effective_gain (before att_in and before output VOA): 21.7 dB
-		o P in: -0.746 dBm
-		o P out: 20.96 dBm
-		o P out/ch: -0.55 dBm
+		o P in: -0.806 dBm
+		o P out: 20.901 dBm
+		o P out/ch: -0.61 dBm
 		o NF: 6.25 dB
 		o Out VOA: 3.0 dB
 		o In VOA: 0 dB
@@ -547,7 +547,7 @@
       <c r="J4" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Roadm roadm Site_D
-	- Actual loss: cband: 17.93, lband: 19.45 dB
+	- Actual loss: cband: 17.93, lband: 19.39 dB
 </t>
         </is>
       </c>
@@ -555,9 +555,9 @@
         <is>
           <t xml:space="preserve">Transceiver trx Site_D
 	- GSNR(0.1nm):: cband: 24.87, lband: 25.37 dB
-	- GSNR(signal bw):: cband: 20.78, lband: 21.29 dB
-	- OSNR ASE (0.1nm):: cband: 25.55, lband: 26.65 dB
-	- OSNR ASE(signal bw):: cband: 21.47, lband: 22.57 dB
+	- GSNR(signal bw):: cband: 20.79, lband: 21.29 dB
+	- OSNR ASE (0.1nm):: cband: 25.55, lband: 26.61 dB
+	- OSNR ASE(signal bw):: cband: 21.47, lband: 22.53 dB
 	- CD:: cband: 4008.00, lband: 4008.00 ps/nm
 	- PMD:: cband: 0.62, lband: 0.62 ps
 	- PDL:: cband: 0.00, lband: 0.00 dB

</xml_diff>